<commit_message>
feat(catalog): add 3 new games to Excel catalog generator
</commit_message>
<xml_diff>
--- a/public/games-catalog.xlsx
+++ b/public/games-catalog.xlsx
@@ -6,7 +6,7 @@
     <sheet name="Catalogue Jeux Ardoise" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Catalogue Jeux Ardoise'!A1:H18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Catalogue Jeux Ardoise'!A1:H21</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:H21"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="24.83203125" customWidth="1"/>
@@ -859,16 +859,16 @@
         <v>17</v>
       </c>
       <c r="B18" t="str">
-        <v>Compteur Universel</v>
+        <v>Mölkky</v>
       </c>
       <c r="C18" t="str">
-        <v>Ardoise libre adaptée à tous vos jeux de société.</v>
+        <v>Faites tomber les quilles en bois numérotées pour marquer des points et atteindre exactement 50 points. Attention au dépassement qui vous renvoie à 25 points et aux 3 lancers ratés consécutifs !</v>
       </c>
       <c r="D18" t="str">
-        <v>https://ardoise.art-crea.fr/jeux/compteur-universel</v>
+        <v>https://ardoise.art-crea.fr/jeux/molkky</v>
       </c>
       <c r="E18" t="str">
-        <v>Tous jeux</v>
+        <v>12 quilles</v>
       </c>
       <c r="F18">
         <v>2</v>
@@ -877,13 +877,91 @@
         <v>12</v>
       </c>
       <c r="H18" t="str">
+        <v>molkky</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Yam's / Yahtzee</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Lancez les 5 dés jusqu’à 3 fois par tour, remplissez les 13 combinaisons de votre grille officielle, visez le bonus de 35 points et le mythique Yam’s à 50 points !</v>
+      </c>
+      <c r="D19" t="str">
+        <v>https://ardoise.art-crea.fr/jeux/yams-yahtzee</v>
+      </c>
+      <c r="E19" t="str">
+        <v>5 dés</v>
+      </c>
+      <c r="F19">
+        <v>2</v>
+      </c>
+      <c r="G19">
+        <v>6</v>
+      </c>
+      <c r="H19" t="str">
+        <v>yams-yahtzee</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Dixit</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Énoncez un indice énigmatique, retrouvez la carte du conteur et bluffez vos adversaires avec vos propres illustrations. Le premier joueur à franchir 30 points l’emporte !</v>
+      </c>
+      <c r="D20" t="str">
+        <v>https://ardoise.art-crea.fr/jeux/dixit</v>
+      </c>
+      <c r="E20" t="str">
+        <v>Jeu illustré</v>
+      </c>
+      <c r="F20">
+        <v>3</v>
+      </c>
+      <c r="G20">
+        <v>8</v>
+      </c>
+      <c r="H20" t="str">
+        <v>dixit</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21">
+        <v>20</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Compteur Universel</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Ardoise libre adaptée à tous vos jeux de société.</v>
+      </c>
+      <c r="D21" t="str">
+        <v>https://ardoise.art-crea.fr/jeux/compteur-universel</v>
+      </c>
+      <c r="E21" t="str">
+        <v>Tous jeux</v>
+      </c>
+      <c r="F21">
+        <v>2</v>
+      </c>
+      <c r="G21">
+        <v>12</v>
+      </c>
+      <c r="H21" t="str">
         <v>compteur-universel</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H18"/>
+  <autoFilter ref="A1:H21"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H18"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H21"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>